<commit_message>
fix: support multi-line walkover scores in bucs data extraction
</commit_message>
<xml_diff>
--- a/data/bucs_data.xlsx
+++ b/data/bucs_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brynprice/uk-football-history/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C04AC54-AA48-4242-818A-82E994A93ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED50DAB-45F3-CC4F-988C-F7AB07B85242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16540" xr2:uid="{1642198C-491C-714F-AF19-53BC029CD0A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="466">
   <si>
     <t>South Eastern Tier 1 - 1A</t>
   </si>
@@ -1269,6 +1269,171 @@
   </si>
   <si>
     <t>6 - 42</t>
+  </si>
+  <si>
+    <t>6 - 6</t>
+  </si>
+  <si>
+    <t>34 - 0</t>
+  </si>
+  <si>
+    <t>13 - 8</t>
+  </si>
+  <si>
+    <t>44 - 0</t>
+  </si>
+  <si>
+    <t>York St John Open 1</t>
+  </si>
+  <si>
+    <t>2 - 18</t>
+  </si>
+  <si>
+    <t>13 - 38</t>
+  </si>
+  <si>
+    <t>28 - 6</t>
+  </si>
+  <si>
+    <t>16 - 0</t>
+  </si>
+  <si>
+    <t>University Of Greenwich, Avery Hill Rd, Eltham, London SE9 2UG Provider: American Football 21-22</t>
+  </si>
+  <si>
+    <t>University Of Greenwich, Avery Hill Rd, Eltham, London SE9 2UG</t>
+  </si>
+  <si>
+    <t>0 - 37</t>
+  </si>
+  <si>
+    <t>Liverpool John Moores Open 1</t>
+  </si>
+  <si>
+    <t>27 - 0</t>
+  </si>
+  <si>
+    <t>JMO Sports Park Blaguegate Playing Fields Liverpool Road Skelmersdale WN8 8BX Provider: American Football 21-22</t>
+  </si>
+  <si>
+    <t>JMO Sports Park Blaguegate Playing Fields Liverpool Road Skelmersdale WN8 8BX</t>
+  </si>
+  <si>
+    <t>8 - 0</t>
+  </si>
+  <si>
+    <t>Cryfield 4G Provider: University of Warwick</t>
+  </si>
+  <si>
+    <t>Cryfield Sports Pavilion, Coventry, UK CV4 7EU Coventry CV4 7AL</t>
+  </si>
+  <si>
+    <t>0 - 25</t>
+  </si>
+  <si>
+    <t>14/12/2025</t>
+  </si>
+  <si>
+    <t>Costello Stadium</t>
+  </si>
+  <si>
+    <t>Anlaby Park Rd N Hull Hull HU4 6XQ</t>
+  </si>
+  <si>
+    <t>18 - 0</t>
+  </si>
+  <si>
+    <t>25/1/2026</t>
+  </si>
+  <si>
+    <t>UEA Colney Lane Playing Fields, Norwich, NR4 7UE Provider: American Football 21-22</t>
+  </si>
+  <si>
+    <t>Norwich, NR4 7UE</t>
+  </si>
+  <si>
+    <t>13 - 20</t>
+  </si>
+  <si>
+    <t>12:15</t>
+  </si>
+  <si>
+    <t>52 - 0</t>
+  </si>
+  <si>
+    <t>20 - 30</t>
+  </si>
+  <si>
+    <t>46 - 0</t>
+  </si>
+  <si>
+    <t>9 - 6</t>
+  </si>
+  <si>
+    <t>Harlington Sports Ground Sipson Lane Harlington Middlesex UB3 5AQ Provider: Cricket 21-22</t>
+  </si>
+  <si>
+    <t>Hayes UB3 5AQ, UK</t>
+  </si>
+  <si>
+    <t>0 - 9</t>
+  </si>
+  <si>
+    <t>37 - 12</t>
+  </si>
+  <si>
+    <t>22 - 49</t>
+  </si>
+  <si>
+    <t>8 - 20</t>
+  </si>
+  <si>
+    <t>36 - 0</t>
+  </si>
+  <si>
+    <t>41 - 0</t>
+  </si>
+  <si>
+    <t>14 - 23</t>
+  </si>
+  <si>
+    <t>20 - 14</t>
+  </si>
+  <si>
+    <t>20 - 26</t>
+  </si>
+  <si>
+    <t>28/1/2026</t>
+  </si>
+  <si>
+    <t>32 - 3</t>
+  </si>
+  <si>
+    <t>01/2/2026</t>
+  </si>
+  <si>
+    <t>56 - 8</t>
+  </si>
+  <si>
+    <t>17 - 7</t>
+  </si>
+  <si>
+    <t>0 - 18</t>
+  </si>
+  <si>
+    <t>0 - 43</t>
+  </si>
+  <si>
+    <t>10 - 7</t>
+  </si>
+  <si>
+    <t>0 - 14</t>
+  </si>
+  <si>
+    <t>33 - 8</t>
+  </si>
+  <si>
+    <t>57 - 7</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D36C6C2A-6236-3A41-9DF0-360A3C916FDF}">
-  <dimension ref="A1:A1561"/>
+  <dimension ref="A1:A2139"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -9452,6 +9617,2896 @@
         <v>2</v>
       </c>
     </row>
+    <row r="1562" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1562" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1563" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1564" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1565" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1566" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1567" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1568" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1569" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1570" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1571" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1572" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1573" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1574" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1575" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1576" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1577" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1578" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1579" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1580" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1581" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1582" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1583" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1584" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1585" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1586" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1587" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1588" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1588" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1589" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1590" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1591" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1592" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1593" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1594" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1595" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1596" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1597" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1598" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1599" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1600" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1601" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1602" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1603" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1604" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1605" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1606" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1607" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1608" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1609" s="1" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1610" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1611" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1612" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1613" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1614" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1615" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1616" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1617" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="1618" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1618" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="1619" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1619" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1620" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1620" s="1" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="1621" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1621" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1622" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1622" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="1623" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1623" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1624" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1624" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1625" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1625" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="1626" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1626" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1627" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1628" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1628" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1629" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1630" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1630" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1631" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1631" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="1632" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1632" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1633" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1633" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="1634" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1634" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1635" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1635" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1636" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1637" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1638" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1639" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1640" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1641" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1642" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1643" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1644" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1645" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1646" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1647" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="1648" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1648" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1649" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1650" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1651" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1652" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1653" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1654" s="1" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1655" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1656" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1657" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1658" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1659" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1660" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1661" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1662" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1663" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1664" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1665" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1666" s="1" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1667" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1668" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1669" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1670" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1671" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1672" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1673" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1674" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1675" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1676" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1677" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1678" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1679" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1680" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1681" s="1" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1682" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1683" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1684" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1685" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1686" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1687" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1688" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1689" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1690" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1691" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1692" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1693" s="1" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1694" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1695" s="1" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1696" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1697" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1698" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1699" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1700" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1700" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1701" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1701" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1702" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1702" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="1703" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1703" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1704" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1704" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="1705" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1705" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1706" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1706" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1707" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1707" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1708" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1708" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1709" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1709" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="1710" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1710" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1711" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="1712" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1712" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1713" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1713" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="1714" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1714" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1715" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1715" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="1716" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1716" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="1717" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1717" s="1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="1718" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1718" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1719" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1719" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1720" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1720" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="1721" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1721" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1722" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1722" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="1723" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1723" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1724" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1724" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="1725" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1725" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="1726" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1726" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="1727" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1727" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="1728" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1728" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="1729" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1729" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1730" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1730" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="1731" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1731" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1732" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1732" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1733" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1733" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="1734" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1734" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="1735" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1735" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1736" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1736" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="1737" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1737" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="1738" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1738" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="1739" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1739" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="1740" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1740" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="1741" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1741" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1742" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1742" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1743" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1743" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1744" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1744" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1745" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1745" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="1746" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1746" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1747" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1747" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1748" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1748" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="1749" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1749" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="1750" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1750" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="1751" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1751" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="1752" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1752" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="1753" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1753" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1754" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1754" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="1755" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1755" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1756" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1756" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1757" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1757" s="1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="1758" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1758" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1759" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1759" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="1760" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1760" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1761" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1761" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="1762" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1762" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1763" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1763" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1764" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1764" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1765" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1765" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1766" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1766" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1767" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1767" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1768" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1768" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="1769" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1769" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1770" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1770" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1771" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1771" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1772" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1772" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="1773" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1773" s="1" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="1774" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1774" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="1775" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1775" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="1776" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1776" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1777" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1777" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="1778" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1778" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="1779" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1779" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1780" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1780" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="1781" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1781" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1782" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1782" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="1783" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1783" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1784" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1784" s="1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="1785" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1785" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="1786" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1786" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1787" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1787" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1788" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1788" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1789" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1789" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="1790" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1790" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1791" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1791" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="1792" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1792" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1793" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1793" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="1794" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1794" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1795" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1795" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1796" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1796" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="1797" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1797" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="1798" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1798" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1799" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1800" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1800" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1801" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="1802" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1802" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1803" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1803" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="1804" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1804" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1805" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1805" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="1806" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1806" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1807" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1807" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1808" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1808" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="1809" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1809" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="1810" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1810" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="1811" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1811" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1812" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1812" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1813" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1813" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1814" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1814" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1815" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1815" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="1816" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1816" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1817" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1817" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="1818" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1818" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1819" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1819" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1820" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1820" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="1821" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1821" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1822" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1822" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1823" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1823" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="1824" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1824" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="1825" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1825" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1826" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1826" s="1" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="1827" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1827" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1828" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1828" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="1829" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1829" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1830" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1830" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1831" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1831" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1832" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1832" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1833" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1833" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1834" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1834" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="1835" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1835" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1836" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1836" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1837" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1837" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="1838" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1838" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1839" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1840" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1841" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1842" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1842" s="1" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="1843" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1843" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="1844" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1844" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1845" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1845" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1846" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1846" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1847" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1847" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1848" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1848" s="1" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="1849" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1849" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1850" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1850" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1851" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1852" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1852" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1853" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1853" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1854" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1854" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="1855" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1855" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1856" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1856" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1857" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1857" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="1858" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1858" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1859" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1859" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="1860" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1860" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1861" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1862" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1862" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1863" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1863" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1864" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1864" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="1865" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1865" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="1866" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1866" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="1867" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1867" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1868" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1868" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1869" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1869" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="1870" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1870" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1871" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1871" s="1" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="1872" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1872" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1873" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1874" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1875" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1876" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1877" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1878" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1879" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1880" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1881" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1882" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1883" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1884" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1885" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1886" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1887" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1888" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1889" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1890" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1891" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1892" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1893" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1894" s="1" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1895" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1896" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1897" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1898" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1899" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="1900" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1900" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="1901" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1901" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1902" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1902" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="1903" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1903" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="1904" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1904" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1905" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1905" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="1906" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1906" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1907" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1907" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1908" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1908" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1909" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1909" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1910" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1910" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="1911" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1911" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="1912" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1912" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1913" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1913" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1914" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1914" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="1915" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1915" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1916" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1916" s="1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="1917" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1917" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1918" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1918" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1919" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1919" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1920" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1920" s="1" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1921" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1921" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1922" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1922" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="1923" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1923" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="1924" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1924" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1925" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1925" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1926" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1926" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="1927" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1927" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1928" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1928" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="1929" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1929" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1930" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1930" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="1931" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1931" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1932" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1932" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="1933" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1933" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="1934" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1934" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="1935" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1935" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="1936" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1936" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1937" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1937" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="1938" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1938" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="1939" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1939" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1940" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1940" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="1941" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1941" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1942" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1942" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1943" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1943" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1944" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1944" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="1945" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1945" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1946" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1946" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="1947" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1947" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1948" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1948" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1949" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1949" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1950" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1950" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="1951" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1951" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1952" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1952" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="1953" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1953" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1954" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1954" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="1955" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1955" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="1956" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1956" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="1957" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1957" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="1958" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1958" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="1959" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1959" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1960" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1960" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1961" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1961" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="1962" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1962" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1963" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1963" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="1964" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1964" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1965" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1965" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="1966" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1966" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="1967" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1967" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="1968" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1968" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="1969" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1969" s="1" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="1970" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1970" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="1971" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1971" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1972" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1972" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="1973" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1973" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1974" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1974" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1975" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1975" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="1976" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1976" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1977" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1977" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1978" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1978" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="1979" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1979" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="1980" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1980" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="1981" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1981" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="1982" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1982" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="1983" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1983" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1984" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1984" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1985" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1985" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="1986" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1986" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1987" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1987" s="1" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="1988" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1988" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1989" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1989" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1990" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1990" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="1991" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1991" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="1992" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1992" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1993" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1993" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1994" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1994" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1995" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1995" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1996" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1996" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="1997" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1997" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1998" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1998" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="1999" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1999" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2000" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2000" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2001" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2001" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2002" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2002" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="2003" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2003" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2004" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2004" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2005" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2005" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2006" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2006" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2007" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2007" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2008" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2008" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="2009" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2009" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2010" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2010" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="2011" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2011" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2012" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2012" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="2013" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2013" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2014" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2014" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="2015" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2015" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2016" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2016" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2017" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2017" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2018" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2018" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2019" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2019" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2020" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2020" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2021" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2021" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="2022" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2022" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2023" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2023" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2024" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2024" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2025" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2025" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2026" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2026" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2027" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2027" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="2028" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2028" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2029" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2029" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2030" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2030" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2031" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2031" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2032" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2032" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2033" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2033" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2034" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2034" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2035" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2035" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="2036" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2036" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2037" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2037" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2038" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2038" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2039" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2039" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2040" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2040" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2041" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2041" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2042" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2042" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2043" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2043" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2044" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2044" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2045" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2045" s="1" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="2046" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2046" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2047" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2047" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2048" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2048" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2049" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2049" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="2050" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2050" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2051" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2051" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="2052" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2052" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2053" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2053" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2054" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2054" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2055" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2055" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2056" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2056" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2057" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2057" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="2058" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2058" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2059" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2059" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2060" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2060" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2061" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2061" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="2062" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2062" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="2063" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2063" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2064" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2064" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="2065" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2065" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2066" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2066" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2067" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2067" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2068" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2068" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2069" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2069" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="2070" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2070" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2071" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2071" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2072" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2072" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2073" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2073" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="2074" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2074" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2075" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2075" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2076" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2076" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2077" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2077" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2078" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2078" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2079" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2079" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2080" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2080" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2081" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2081" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2082" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2082" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2083" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2083" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2084" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2084" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2085" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2085" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="2086" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2086" s="1" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="2087" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2087" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="2088" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2088" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="2089" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2089" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2090" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2090" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2091" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2091" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2092" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2092" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2093" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2093" s="1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="2094" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2094" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2095" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2095" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2096" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2096" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2097" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2097" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2098" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2098" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="2099" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2099" s="1" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="2100" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2100" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="2101" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2101" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2102" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2102" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2103" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2103" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2104" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2104" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2105" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2105" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2106" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2106" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2107" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2107" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2108" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2108" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2109" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2109" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2110" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2110" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2111" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2111" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="2112" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2112" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="2113" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2113" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="2114" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2114" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2115" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2115" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2116" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2116" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2117" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2117" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2118" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2118" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="2119" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2119" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2120" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2120" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2121" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2121" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2122" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2122" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2123" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2123" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2124" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2124" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2125" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2125" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="2126" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2126" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2127" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2127" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2128" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2128" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2129" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2129" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2130" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2130" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2131" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2131" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2132" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2132" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2133" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2133" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="2134" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2134" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="2135" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2135" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2136" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2136" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2137" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2137" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2138" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2138" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2139" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2139" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: resolve team aliases in standings, career timeline, and awards
</commit_message>
<xml_diff>
--- a/data/bucs_data.xlsx
+++ b/data/bucs_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brynprice/uk-football-history/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA10E49-F7F3-424F-95FD-A0E9EE01278E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4681AEA2-D274-974E-A241-52D8169AF37D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16520" xr2:uid="{1642198C-491C-714F-AF19-53BC029CD0A7}"/>
   </bookViews>
@@ -36,165 +36,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="163">
-  <si>
-    <t>Brighton Open 1</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="262">
   <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Southern Tier 1 - 1A</t>
   </si>
   <si>
-    <t>Oxford Open 1</t>
-  </si>
-  <si>
-    <t>Tilsley Park 3G Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Dunmore Rd, Abingdon OX14 1PU</t>
-  </si>
-  <si>
-    <t>Parking available. Players must wear appropriate rugby and football boots only. No metal blades or spikes are allowed. Please ensure all footwear is clean before using the pitch. Athletes can walk across the 4G pitch (when it is not in use by others) with training shoes and use the 5m safety run off zone around the pitch when wearing training shoes (no spikes). No football, rugby or similar boots are to be worn on the track except whilst crossing to access the infield 4G pitch.</t>
-  </si>
-  <si>
-    <t>King's College Open 1</t>
-  </si>
-  <si>
-    <t>Portsmouth Open 1</t>
-  </si>
-  <si>
-    <t>SGS Open 1</t>
-  </si>
-  <si>
-    <t>Bournemouth Open 1</t>
-  </si>
-  <si>
-    <t>Bournemouth University Sports Campus, Chapel Gate, Christchurch, BH23 6BL Provider: Football 21-22</t>
+    <t>South Western Tier 2 - 2A</t>
   </si>
   <si>
     <t>Bournemouth University Sports Campus, Chapel Gate, Christchurch, BH23 6BL</t>
   </si>
   <si>
-    <t>Grass pitches. Free parking available. First aid provision: LUL-MED Services Ltd (minimum first aid at work). Defibrillator on site. Please visit reception in the club house on arrival for changing room keys – cash deposit required. Please note only food and drink purchased from the bar to be consumed on site, no alcohol to be brought onto site.</t>
-  </si>
-  <si>
-    <t>Hertfordshire Open 1</t>
-  </si>
-  <si>
-    <t>Birmingham Open 1</t>
-  </si>
-  <si>
-    <t>Leeds Beckett Open 1</t>
-  </si>
-  <si>
-    <t>Nottingham Open 1</t>
-  </si>
-  <si>
-    <t>West Park Rugby Club, The Sycamores, Bramhope, Leeds LS16 9JR Provider: Rugby Union 21-22</t>
-  </si>
-  <si>
     <t>West Park Rugby Club, The Sycamores, Bramhope, Leeds LS16 9JR</t>
   </si>
   <si>
-    <t>Edinburgh Open 1</t>
-  </si>
-  <si>
-    <t>Glasgow Open 1</t>
-  </si>
-  <si>
-    <t>0 - 6</t>
-  </si>
-  <si>
-    <t>Nottingham Open 2</t>
-  </si>
-  <si>
-    <t>Sheffield Hallam Open 1</t>
-  </si>
-  <si>
-    <t>3G, David Ross Sports Centre (DRSV), Beeston Lane, Nottingham. NG7 2RJ Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>3G, David Ross Sports Centre (DRSV), Beeston Lane, Nottingham. NG7 2RJ Nottingham NG7 2RD</t>
-  </si>
-  <si>
-    <t>Warwick Open 1</t>
-  </si>
-  <si>
-    <t>Kent Open 1</t>
-  </si>
-  <si>
-    <t>Imperial Open 1</t>
-  </si>
-  <si>
-    <t>Brunel Open 1</t>
-  </si>
-  <si>
-    <t>Exeter Open 1</t>
-  </si>
-  <si>
-    <t>Site 5, Sports Park, Kingston Lane, Uxbridge, UB8 3PH Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Site 5, Sports Park, Kingston Lane, Uxbridge, UB8 3PH Uxbridge UB8 3PH</t>
-  </si>
-  <si>
-    <t>Site 5 is a 5 minute walk from the sports park. You will be able to park at the sports park, make sure you ask for a visitor permit from the sport pavilion staff. As you leave the sports park, you will need to make a left on Kingston Lane. At end of the road, turn right onto Pield Heath Road. Site 5 is located on the left hand side, at the end of the row of houses - you will see the gate as you approach. Please do not use the residents driveway to drop off equipment.</t>
-  </si>
-  <si>
-    <t>Greenwich Open 1</t>
-  </si>
-  <si>
-    <t>Royal Holloway Open 1</t>
-  </si>
-  <si>
-    <t>Cardiff Open 1</t>
-  </si>
-  <si>
-    <t>UWE Open 1</t>
-  </si>
-  <si>
-    <t>Manchester Open 1</t>
-  </si>
-  <si>
-    <t>Liverpool Open 1</t>
-  </si>
-  <si>
-    <t>Sports &amp; Exercise Peffermill Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>42 Peffermill Road, EH16 5LL</t>
-  </si>
-  <si>
-    <t>Time on BUCS Play is start time. Side pitches will be available for pre-match warm ups.</t>
-  </si>
-  <si>
-    <t>Durham Open 1</t>
-  </si>
-  <si>
-    <t>Surrey Open 1</t>
+    <t>Boots must be worn, no trainers allowed Access 30 minutes before start time</t>
+  </si>
+  <si>
+    <t>Midlands Tier 2 - 2A</t>
+  </si>
+  <si>
+    <t>Coldhams Common (Abbey Pools), Whitehall Road CB5 8NT</t>
+  </si>
+  <si>
+    <t>Minibus and Coaches drop-off only. Then Park at the Designer Outlet on A64. Cars to Park in Pay and Display Parking on campus.</t>
+  </si>
+  <si>
+    <t>University of Brighton Falmer campus, Village Way, Brighton, UK BN1 9PH</t>
+  </si>
+  <si>
+    <t>South Eastern Tier 2 - 2A</t>
+  </si>
+  <si>
+    <t>71 Holland Rd, London E15 3BP, UK</t>
+  </si>
+  <si>
+    <t>Southern Tier 2 - 2A</t>
+  </si>
+  <si>
+    <t>Northern Tier 1 - 1A</t>
+  </si>
+  <si>
+    <t>DMU/Beaumont Park Football Club, Leicester LE4 1ES</t>
   </si>
   <si>
     <t>20 - 0</t>
   </si>
   <si>
-    <t>Queen Mary Open 1</t>
-  </si>
-  <si>
-    <t>Loughborough Open 1</t>
-  </si>
-  <si>
-    <t>Stirling Open 1</t>
-  </si>
-  <si>
-    <t>Manchester Met Open 1</t>
-  </si>
-  <si>
-    <t>JMO Sports Park Provider: American Football 21-22</t>
+    <t>Chislehurst BR7 6SD, UK</t>
+  </si>
+  <si>
+    <t>No metal studs permitted. A small amount of parking is available for cars and people carriers at the Sports Centre but minibuses must park at The Residences. Please take the first road on the left after entering the campus and follow the round round to the car parks on the right hand side.</t>
   </si>
   <si>
     <t>Blaguegate Playing Fields, Liverpool Road, Skelmersdale WN8 8BX</t>
@@ -203,67 +98,28 @@
     <t>4g Pitch</t>
   </si>
   <si>
-    <t>East Anglia Open 1</t>
-  </si>
-  <si>
-    <t>UWE Open 2</t>
-  </si>
-  <si>
-    <t>Sheffield Open 1</t>
-  </si>
-  <si>
-    <t>Sheffield Hallam University Sports Park (3G) Provider: American Football 21-22</t>
-  </si>
-  <si>
     <t>Sheffield Hallam University Sports Park, Bawtry Road, Sheffield, UK</t>
   </si>
   <si>
     <t>Car – the grounds are located on Bawtry Road (A631 towards Bawtry) approximately one mile from M1 Junction 34 at the south end of the Tinsley viaduct. There is plenty of car parking alongside the main building. Bus – take the x3 (limited service) or 72 bus from Sheffield city centre (bus station or Arundel Gate).</t>
   </si>
   <si>
-    <t>54 - 0</t>
-  </si>
-  <si>
-    <t>Parkwood 3GX, Parkwood, University of Kent, Canterbury, CT2 7SR Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Parkwood 3GX, Parkwood, University of Kent, Canterbury, CT2 7SR CT2 7SR</t>
+    <t>Free Parking</t>
   </si>
   <si>
     <t>Changing facilities in the Pavilion</t>
   </si>
   <si>
-    <t>Edinburgh Napier Open 1</t>
-  </si>
-  <si>
-    <t>Nottingham Trent Open 1</t>
-  </si>
-  <si>
-    <t>Hillside Gardens, Filton Road, BS16 1QG Provider: American Football 21-22</t>
-  </si>
-  <si>
     <t>Hillside Gardens, Filton Road, BS16 1QG</t>
   </si>
   <si>
-    <t>4G Astro pitch. Please wear appropriate footwear. Parking Available.</t>
-  </si>
-  <si>
-    <t>Holywell Rubber Crumb, Loughborough University, LE11 3QF Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Holywell Rubber Crumb, Loughborough University, LE11 3TU Loughborough LE11 3TU</t>
-  </si>
-  <si>
-    <t>Sat Nav - Use LE11 3QF for exact location. Changing in University Stadium.</t>
-  </si>
-  <si>
-    <t>0 - 12</t>
-  </si>
-  <si>
-    <t>Lincoln Open 1</t>
-  </si>
-  <si>
-    <t>Newcastle Open 1</t>
+    <t>3G, Coombe Dingle Sports Complex, Coombe Lane, Bristol BS9 2BJ</t>
+  </si>
+  <si>
+    <t>-No alcohol to be brought on site (bar open for purchasing drinks in line with site license) -Please use appropriate footwear for the 3G (studs must be worn) including coaching staff -Free parking on-site -First aid provision - Community Paramedics. Please report to First Aid room if any issues -£10 deposit required for changing rooms (card payment only) -Please get in touch 7 days prior to your fixture if you would like to pre-order food as an away team</t>
+  </si>
+  <si>
+    <t>24 - 0</t>
   </si>
   <si>
     <t>0 - 0</t>
@@ -272,39 +128,24 @@
     <t>Walkover</t>
   </si>
   <si>
-    <t>Grass and 4G pitches - Please note our Car parking is pay and display.</t>
-  </si>
-  <si>
-    <t>Harlington Sports GroundSipson LaneHarlingtonMiddlesexUB3 5AQ Provider: Rugby Union 21-22</t>
-  </si>
-  <si>
-    <t>Harlington Sports GroundSipson LaneHarlingtonMiddlesexUB3 5AQ UB3 5AQ</t>
-  </si>
-  <si>
-    <t>Free parking at venue</t>
-  </si>
-  <si>
-    <t>Cochrane Park 3G Etherstone Avenue NE7 7JX Provider: Football 21-22</t>
-  </si>
-  <si>
-    <t>Cochrane Park 3G Etherstone Avenue NE7 7JX Newcastle upon Tyne NE7 7JX</t>
+    <t>.</t>
+  </si>
+  <si>
+    <t>Car parking on site</t>
+  </si>
+  <si>
+    <t>0 - 20</t>
   </si>
   <si>
     <t>12:30</t>
   </si>
   <si>
+    <t>6 - 13</t>
+  </si>
+  <si>
     <t>15:00</t>
   </si>
   <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>10:00</t>
-  </si>
-  <si>
     <t>11:00</t>
   </si>
   <si>
@@ -320,211 +161,667 @@
     <t>13:30</t>
   </si>
   <si>
-    <t>35 - 0</t>
-  </si>
-  <si>
-    <t>Clifton Sports Hub Grass Pitch 1, Clifton Campus, Nottingham NG11 8NS Provider: Rugby League 21-22</t>
+    <t>7 - 14</t>
+  </si>
+  <si>
+    <t>0 - 29</t>
   </si>
   <si>
     <t>Nottingham Trent University, Clifton Campus, Clifton Lane, Clifton, Nottingham, UK</t>
   </si>
   <si>
-    <t>Entry at North Gate (main entrance) drop off at coach stop and walk. No drop off outside sports centre. No parking for coaches on campus.</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Staffordshire Open 1</t>
-  </si>
-  <si>
-    <t>University Of Greenwich, Avery Hill Rd, Eltham, London SE9 2UG Provider: American Football 21-22</t>
+    <t>10 - 0</t>
+  </si>
+  <si>
+    <t>Sir Stanley Matthews Sports Centre, Staffordshire University, Leek Road, Stoke on Trent. ST4 2DF</t>
+  </si>
+  <si>
+    <t>Playing Fields. - Coach parking is limited on campus. All driver's must report to the Sports Centre reception to validate their parking.</t>
+  </si>
+  <si>
+    <t>6 - 12</t>
+  </si>
+  <si>
+    <t>6 - 14</t>
+  </si>
+  <si>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>20 - 6</t>
+  </si>
+  <si>
+    <t>14:30</t>
   </si>
   <si>
     <t>University Of Greenwich, Avery Hill Rd, Eltham, London SE9 2UG</t>
   </si>
   <si>
-    <t>27 - 0</t>
-  </si>
-  <si>
-    <t>41 - 0</t>
-  </si>
-  <si>
-    <t>32 - 3</t>
-  </si>
-  <si>
-    <t>6 - 7</t>
-  </si>
-  <si>
-    <t>UCLan Open 1</t>
-  </si>
-  <si>
-    <t>34 - 12</t>
-  </si>
-  <si>
-    <t>13:45</t>
-  </si>
-  <si>
-    <t>Oxford Brookes Open 1</t>
-  </si>
-  <si>
-    <t>6 - 31</t>
-  </si>
-  <si>
-    <t>Royal Holloway Grass Pitches - Eastfields Provider: Rugby Union 21-22</t>
+    <t>JMO Sports Park Blaguegate Playing Fields Liverpool Road Skelmersdale WN8 8BX</t>
+  </si>
+  <si>
+    <t>0 - 25</t>
+  </si>
+  <si>
+    <t>Norwich, NR4 7UE</t>
+  </si>
+  <si>
+    <t>36 - 0</t>
+  </si>
+  <si>
+    <t>York St John University Sports Fields, Haxby Rd, New Earswick, York YO31 8FY, UK</t>
+  </si>
+  <si>
+    <t>32 - 8</t>
+  </si>
+  <si>
+    <t>33 - 12</t>
+  </si>
+  <si>
+    <t>26 - 0</t>
+  </si>
+  <si>
+    <t>21 - 6</t>
+  </si>
+  <si>
+    <t>48 - 0</t>
+  </si>
+  <si>
+    <t>16 - 7</t>
+  </si>
+  <si>
+    <t>University of Warwick, Cryfield Sports Pavilion, Coventry CV4 7AL, UK</t>
+  </si>
+  <si>
+    <t>PLEASE NOTE THERE IS NO PARKING FOR COACHES or MINIBUSES AT ANY OF OUR VENUES. CAR PARKING IS EXTREMELY LIMITED AND WE CANNOT GUARANTEE SPACES FOR ANY VISITING TEAMS. APOLOGIES. Please can you also remind your students not to park in the Cats and Dogs home next door to campus as this is private property.</t>
   </si>
   <si>
     <t>Royal Holloway Sport, Prune Hill, Egham, TW20 9TR</t>
   </si>
   <si>
-    <t>Royal Holloway Sports Centre can NOT be accessed by car from the main campus. Teams will need to drive to the Sports Centre using the postcode here. We have a limited number of car parking spaces, and no coach parking. We operate a number plate recognition scheme on campus – all teams wishing to park on campus need to register their vehicle at the Sports Centre Reception. Please allow extra time before your fixtures to do this. All times listed for home matches are the start time of the match, except for volleyball, where this is the start of the official warm up. Royal Holloway teams play in green and purple.</t>
-  </si>
-  <si>
-    <t>8 - 21</t>
-  </si>
-  <si>
-    <t>14 - 18</t>
-  </si>
-  <si>
-    <t>6 - 8</t>
+    <t>50 - 6</t>
+  </si>
+  <si>
+    <t>28 - 0</t>
+  </si>
+  <si>
+    <t>0 - 36</t>
   </si>
   <si>
     <t>15:30</t>
   </si>
   <si>
-    <t>National Trophy</t>
-  </si>
-  <si>
-    <t>SGS WISE Campus Provider: SGS College</t>
-  </si>
-  <si>
-    <t>Stoke Gifford, Bristol BS34 8LP, UK</t>
-  </si>
-  <si>
-    <t>Northern Conference Cup</t>
-  </si>
-  <si>
-    <t>Southern Conference Cup</t>
-  </si>
-  <si>
-    <t>National Championship</t>
-  </si>
-  <si>
-    <t>Bournbrook 3G Provider: American Football 21-22</t>
+    <t>Midlands Tier 1 - 1A</t>
+  </si>
+  <si>
+    <t>0 - 48</t>
+  </si>
+  <si>
+    <t>Northern Tier 2 - 2A</t>
   </si>
   <si>
     <t>University of Birmingham, Birmingham B15 2TT, UK</t>
   </si>
   <si>
-    <t>15 - 6</t>
-  </si>
-  <si>
-    <t>42 - 6</t>
-  </si>
-  <si>
-    <t>8 - 24</t>
-  </si>
-  <si>
-    <t>51 - 0</t>
-  </si>
-  <si>
-    <t>28 - 10</t>
-  </si>
-  <si>
-    <t>Langstone 3G Pitch, Furze Lane, Southsea PO4 8LW Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Langstone Grass Pitch, Furze Lane, Southsea PO4 8LW Portsmouth Southsea PO4</t>
-  </si>
-  <si>
-    <t>3G Pitch *(American Football Bookings have 12 Warm Up with a 2pm Start)</t>
-  </si>
-  <si>
-    <t>Platt Lane Provider: MMU Sport</t>
-  </si>
-  <si>
-    <t>M14 7UU Manchester M14 7UU</t>
-  </si>
-  <si>
-    <t>28 - 21</t>
-  </si>
-  <si>
-    <t>15 - 0</t>
-  </si>
-  <si>
-    <t>14 - 12</t>
-  </si>
-  <si>
-    <t>Surrey Sports Park GU2 7AD Provider: American Football 21-22</t>
-  </si>
-  <si>
-    <t>Surrey Sports Park, Richard Meyjes Road, Guildford GU2 7AD, UK</t>
-  </si>
-  <si>
-    <t>Parking free up to 3 hours. Students staying for longer will need to give their registration number at reception to be exempt from parking fines.</t>
-  </si>
-  <si>
-    <t>43 - 38</t>
-  </si>
-  <si>
-    <t>26/2/2022</t>
+    <t>Inglemire Lane, Hull HU6 8JG, UK</t>
+  </si>
+  <si>
+    <t>21 - 0</t>
+  </si>
+  <si>
+    <t>Langon Lane, Nackington Road, Canterbury Kent CT4 7AS</t>
+  </si>
+  <si>
+    <t>12 - 28</t>
+  </si>
+  <si>
+    <t>6 - 36</t>
+  </si>
+  <si>
+    <t>12 - 18</t>
+  </si>
+  <si>
+    <t>Borders Tier 2 - 2A</t>
+  </si>
+  <si>
+    <t>Olympia Building Middlesbrough TS1 3BF</t>
+  </si>
+  <si>
+    <t>No parking available</t>
+  </si>
+  <si>
+    <t>8 - 13</t>
+  </si>
+  <si>
+    <t>2 - 22</t>
+  </si>
+  <si>
+    <t>6 - 9</t>
+  </si>
+  <si>
+    <t>32 - 0</t>
+  </si>
+  <si>
+    <t>We have a limited number of car parking spaces, and no coach parking. We operate a number plate recognition scheme on campus – all teams wishing to park on campus need to register their vehicle at the Sports Centre Reception. Please allow extra time before your fixtures to do this. All times listed for home matches are the start time of the match, except for volleyball, where this is the start of the official warm up. Royal Holloway teams play in green and purple.</t>
+  </si>
+  <si>
+    <t>Grass pitches. Free parking available. First aid provision: Defibrillator on site. Please visit reception in the club house on arrival for changing room keys – cash deposit required.</t>
+  </si>
+  <si>
+    <t>Gannochy 3G Astro Gannochy Sports Centre FK9 4LA</t>
+  </si>
+  <si>
+    <t>Edge Hill University, Saint Helens Road, Ormskirk, L39 4QP UK</t>
+  </si>
+  <si>
+    <t>Druid Park, Woolsington, Newcastle upon Tyne, NE13 8DF, UK</t>
+  </si>
+  <si>
+    <t>Ample parking available on site. 3G pitch so please ensure your team wear the correct footwear.</t>
+  </si>
+  <si>
+    <t>• Address – DMU/Beaumont Park Football Club, Leicester LE4 1ES • Playing Surface – Artificial rubber crumb • Parking - There is parking available on site, however this is limited. • Members of staff will be present at all facilities. Please report accidents or near misses to these members of staff as soon as possible. • This team play’s in predominantly Red kit, and if you foresee a clash please let me know asap.</t>
+  </si>
+  <si>
+    <t>Garscube Sports Complex, West of Scotland Science Park, Maryhill Road, Glasgow. G20 0SP (01413305363)</t>
+  </si>
+  <si>
+    <t>Parking for buses, vending machines only, footwear policy for football on 3g pitch - no blades of any kind allowed on this pitch. If teams turn up with incorrect footwear they will not be allowed to participate. Rubber/moulded studs and astroturf trainers only permitted. All Lacrosse/American Football fixtures take place on synthetic pitch 1 which is sand dressed synthetic pitch, suitable footwear for this pitch is astro trainers or rubber moulded studs - no blades allowed</t>
+  </si>
+  <si>
+    <t>Laisteridge Lane, Bradford, UK</t>
+  </si>
+  <si>
+    <t>Postcode:BD5 0NH All visiting Universities MUST park in the main car park at the back of Dennis Bellamy Halls opposite the astroturf to avoid being clamped. If you require a parking slot you will need a permit. Please email G.Zinonos1@bradford.ac.uk to arrange this, you will need a vehicle registration. PLEASE NOTE METAL STUDS AND BLADES ARE NOT ALLOWED.</t>
+  </si>
+  <si>
+    <t>[Clifton Campus Grass Pitch 1, Nottingham Trent Clifton Campus, NG11 8NS]</t>
   </si>
   <si>
     <t>9 - 0</t>
   </si>
   <si>
-    <t>27/2/2022</t>
-  </si>
-  <si>
-    <t>31 - 6</t>
-  </si>
-  <si>
-    <t>23 - 7</t>
-  </si>
-  <si>
-    <t>43 - 2</t>
-  </si>
-  <si>
-    <t>52 - 6</t>
-  </si>
-  <si>
-    <t>Sport &amp; Exercise Peffermill, 3G 1 Provider: The Burgh Varsity</t>
-  </si>
-  <si>
-    <t>42 Peffermill Road, Edinburgh EH16 5LL, UK</t>
-  </si>
-  <si>
-    <t>Time on BUCS is for warm ups, match will start at 1430</t>
-  </si>
-  <si>
-    <t>06/3/2022</t>
-  </si>
-  <si>
-    <t>15 - 23</t>
-  </si>
-  <si>
-    <t>15 - 7</t>
-  </si>
-  <si>
-    <t>3 - 22</t>
-  </si>
-  <si>
-    <t>13/3/2022</t>
-  </si>
-  <si>
-    <t>21 - 12</t>
-  </si>
-  <si>
-    <t>22/3/2022</t>
-  </si>
-  <si>
-    <t>19:45</t>
-  </si>
-  <si>
-    <t>19 - 37</t>
-  </si>
-  <si>
-    <t>27/3/2022</t>
+    <t>Yorkshire Tier 1 - 1A</t>
+  </si>
+  <si>
+    <t>Leeds Mixed 1</t>
+  </si>
+  <si>
+    <t>43 - 19</t>
+  </si>
+  <si>
+    <t>Sheffield Mixed 1</t>
+  </si>
+  <si>
+    <t>02/11/2019</t>
+  </si>
+  <si>
+    <t>West Park Leeds RUFC, The Sycamores, Bramhope, Leeds LS16 9JR, Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Canterbury CC Mixed 1</t>
+  </si>
+  <si>
+    <t>17 - 2</t>
+  </si>
+  <si>
+    <t>City Mixed 1</t>
+  </si>
+  <si>
+    <t>Simon Langon School For Boys Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Loughborough Mixed 1</t>
+  </si>
+  <si>
+    <t>9 - 30</t>
+  </si>
+  <si>
+    <t>Derby Mixed 1</t>
+  </si>
+  <si>
+    <t>03/11/2019</t>
+  </si>
+  <si>
+    <t>Holywell Rubber Crumb, Loughborough University, LE11 3TU Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Holywell Rubber Crumb, Loughborough University, LE11 3TU</t>
+  </si>
+  <si>
+    <t>Changing Rooms at Holywell Stadium</t>
+  </si>
+  <si>
+    <t>South West Tier 1 - 1A</t>
+  </si>
+  <si>
+    <t>Southampton Mixed 1</t>
+  </si>
+  <si>
+    <t>Bath Mixed 1</t>
+  </si>
+  <si>
+    <t>Wide Lane Sports Grounds, Wide Lane, Eastleigh, Hampshire, SO50 5PE Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Wide Lane Sports Grounds, Wide Lane, Eastleigh, Hampshire, SO50 5PE</t>
+  </si>
+  <si>
+    <t>Edge Hill Mixed 1</t>
+  </si>
+  <si>
+    <t>Lancaster Mixed 1</t>
+  </si>
+  <si>
+    <t>Edge Hill Sports Centre, St Helens Road, L39 4QP Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>King's College Mixed 1</t>
+  </si>
+  <si>
+    <t>East London Mixed 1</t>
+  </si>
+  <si>
+    <t>University Of Greenwich, Avery Hill Rd, Eltham, London SE9 2UG Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Chester: Chester Mixed 1</t>
+  </si>
+  <si>
+    <t>Leicester Mixed 1</t>
+  </si>
+  <si>
+    <t>University of Chester, Warrington Campus Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>University of Chester, Warrington Campus, Crab Lane, Warrington, WA2 0DB</t>
+  </si>
+  <si>
+    <t>Grass pitches</t>
+  </si>
+  <si>
+    <t>UWE Mixed 2</t>
+  </si>
+  <si>
+    <t>0 - 33</t>
+  </si>
+  <si>
+    <t>Solent Mixed 1</t>
+  </si>
+  <si>
+    <t>Hillside Gardens, Filton Road, BS16 1QG Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>3G Pitches Only - Please wear appropriate footwear | Parking Available</t>
+  </si>
+  <si>
+    <t>Bournemouth Mixed 1</t>
+  </si>
+  <si>
+    <t>47 - 0</t>
+  </si>
+  <si>
+    <t>Bath Spa Mixed 1</t>
+  </si>
+  <si>
+    <t>Bournemouth University Sports Campus, Chapel Gate, Christchurch, BH23 6BL Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Bristol Mixed 1</t>
+  </si>
+  <si>
+    <t>38 - 11</t>
+  </si>
+  <si>
+    <t>Plymouth Mixed 1</t>
+  </si>
+  <si>
+    <t>3G, Coombe Dingle Sports Complex, Coombe Lane, Bristol BS9 2BJ Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Glasgow Mixed 1</t>
+  </si>
+  <si>
+    <t>17 - 12</t>
+  </si>
+  <si>
+    <t>Heriot-Watt Mixed 1</t>
+  </si>
+  <si>
+    <t>Garscube Sports Complex, West of Scotland Science Park, Maryhill Road, Glasgow. G20 0SP (01413305363) Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Premier - North</t>
+  </si>
+  <si>
+    <t>Nottingham Mixed 1</t>
+  </si>
+  <si>
+    <t>Stirling Mixed 1</t>
+  </si>
+  <si>
+    <t>3G, David Ross Sports Centre (DRSV), Beeston Lane, Nottingham. NG7 2RJ Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>3G, David Ross Sports Centre (DRSV), Beeston Lane, Nottingham. NG7 2RJ</t>
+  </si>
+  <si>
+    <t>Warwick Mixed 1</t>
+  </si>
+  <si>
+    <t>11 - 7</t>
+  </si>
+  <si>
+    <t>Nottingham Trent Mixed 1</t>
+  </si>
+  <si>
+    <t>American Football Pitch - Cryfield Pavilion, University of Warwick Coventry CV4 7AL Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Royal Holloway Mixed 1</t>
+  </si>
+  <si>
+    <t>Brighton Mixed 1</t>
+  </si>
+  <si>
+    <t>Royal Holloway Grass Pitches - Eastfields Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>York St John Mixed 1</t>
+  </si>
+  <si>
+    <t>42 - 20</t>
+  </si>
+  <si>
+    <t>UWS Mixed 1</t>
+  </si>
+  <si>
+    <t>YSJ Haxby Road (GRASS) Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Staffordshire Mixed 1</t>
+  </si>
+  <si>
+    <t>Huddersfield Mixed 1</t>
+  </si>
+  <si>
+    <t>Sir Stanley Matthews Sports Centre - Playing fields, Staffordshire University, Leek Road, Stoke on Trent. ST4 2DF Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Kingston Mixed 1</t>
+  </si>
+  <si>
+    <t>Winchester Mixed 1</t>
+  </si>
+  <si>
+    <t>Tolworth Court Sports Ground, Old Kingston Rd, Worcester Park, KT4 7QH Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Tolworth Court Sports Ground, Old Kingston Rd, Worcester Park, KT4 7QH</t>
+  </si>
+  <si>
+    <t>Northumbria Mixed 1</t>
+  </si>
+  <si>
+    <t>Hull Mixed 1</t>
+  </si>
+  <si>
+    <t>Druid Park, Woolsington, NE13 8DF Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>UCLan Mixed 1</t>
+  </si>
+  <si>
+    <t>8 - 32</t>
+  </si>
+  <si>
+    <t>Sheffield Hallam Mixed 1</t>
+  </si>
+  <si>
+    <t>3G Pitch UCLan Sports Arena Tom Benson Way Preston PR2 1SG Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>3G Pitch UCLan Sports Arena Tom Benson Way Preston PR2 1SG</t>
+  </si>
+  <si>
+    <t>South Eastern 1A - 1A</t>
+  </si>
+  <si>
+    <t>Kent Mixed 1</t>
+  </si>
+  <si>
+    <t>42 - 14</t>
+  </si>
+  <si>
+    <t>Imperial Mixed 1</t>
+  </si>
+  <si>
+    <t>Parkwood 3GX, Parkwood, University of Kent, Canterbury, CT2 7SR Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Parkwood 3GX, Parkwood, University of Kent, Canterbury, CT2 7SR</t>
+  </si>
+  <si>
+    <t>Leeds Beckett Mixed 1</t>
+  </si>
+  <si>
+    <t>Coventry Mixed 1</t>
+  </si>
+  <si>
+    <t>West Park Rugby Club, The Sycamores, Bramhope, Leeds LS16 9JR Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Edinburgh Mixed 1</t>
+  </si>
+  <si>
+    <t>Newcastle Mixed 1</t>
+  </si>
+  <si>
+    <t>Sport &amp; Exercise Peffermill, 3G 1, 42 Peffermill Road,EH16 5LL Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Sport &amp; Exercise Peffermill, 3G 1, 42 Peffermill Road,EH16 5LL</t>
+  </si>
+  <si>
+    <t>Premier - South</t>
+  </si>
+  <si>
+    <t>UWE Mixed 1</t>
+  </si>
+  <si>
+    <t>Hertfordshire Mixed 1</t>
+  </si>
+  <si>
+    <t>Swansea Mixed 1</t>
+  </si>
+  <si>
+    <t>East Anglia Mixed 1</t>
+  </si>
+  <si>
+    <t>American FootballLlandarcy Academy of SportLlandarcy Park,Llandarcy,Neath,Neath Port Talbot.SA10 6JD Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Llandarcy Academy of Sport, Llandarcy Park, Llandarcy, Skewen, Neath, Neath Port Talbot SA10 6JD, UK</t>
+  </si>
+  <si>
+    <t>3G Surface Web: http://www.llandarcyacademy.com t: 01639 648680</t>
+  </si>
+  <si>
+    <t>Reading Mixed 1</t>
+  </si>
+  <si>
+    <t>Portsmouth Mixed 1</t>
+  </si>
+  <si>
+    <t>09/11/2019</t>
+  </si>
+  <si>
+    <t>Reading University Sports Park Whiteknights Campus Reading RG6 6UR Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Reading University Sports Park Whiteknights Campus Reading RG6 6UR</t>
+  </si>
+  <si>
+    <t>Birmingham Mixed 1</t>
+  </si>
+  <si>
+    <t>Bournbrook 3G Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Liverpool Mixed 1</t>
+  </si>
+  <si>
+    <t>Bangor Mixed 1</t>
+  </si>
+  <si>
+    <t>10/11/2019</t>
+  </si>
+  <si>
+    <t>JMO Sports Park Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>10 - 30</t>
+  </si>
+  <si>
+    <t>Gannochy 3G Astro Gannochy Sports Centre FK9 4LA Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>York Mixed 1</t>
+  </si>
+  <si>
+    <t>University of York, YO10 5DD, 22 Acres. Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>University of York, YO10 5DD, 22 Acres.</t>
+  </si>
+  <si>
+    <t>7 - 36</t>
+  </si>
+  <si>
+    <t>Durham Mixed 1</t>
+  </si>
+  <si>
+    <t>Sunderland Mixed 1</t>
+  </si>
+  <si>
+    <t>Robertson Sports Centre, Caplethill Rd, Paisley PA2 7TR Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Caplethill Rd, Paisley PA2 7TR</t>
+  </si>
+  <si>
+    <t>Uni of Hull Sport Park, West Campus pitches Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>UEA Colney Lane Playing Fields, Norwich, NR4 7UE Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Colney Lane Car Park is out of action until middle of November. Closest car park is Triangle Car Park £1.50 NR4 7UE is the closest postcode to Colney Lane - Link is below: https://www.google.com/maps/place/UEA+Colney+Playing+Fields/@52.6221788,1.2227963,17z/data=!3m1!4b1!4m5!3m4!1s0x47d9e0d7f8fbf8ff:0x8dd4656e59f03477!8m2!3d52.6221788!4d1.224985</t>
+  </si>
+  <si>
+    <t>De Montfort Mixed 1</t>
+  </si>
+  <si>
+    <t>Beaumont Park (3G Pitch) Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Clifton Campus Pitch 1 Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Worcester Mixed 1</t>
+  </si>
+  <si>
+    <t>STV Rugby Pitch 1: Sports Training Village, University of Bath, Claverton Down Road, Combe Down, Bath, BA2 7AY UK Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Sports Training Village, University of Bath, Claverton Down Road, Combe Down, Bath, BA2 7AY UK</t>
+  </si>
+  <si>
+    <t>Exeter Mixed 1</t>
+  </si>
+  <si>
+    <t>Cardiff Mixed 1</t>
+  </si>
+  <si>
+    <t>University of Duckes Meadow Sports Field Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Salmonpool Lane, Exeter EX2 4SN, UK</t>
+  </si>
+  <si>
+    <t>There is very limited parking available at Duckes Meadow, please contact aubucs@exeter.ac.uk if you wish to park there.</t>
+  </si>
+  <si>
+    <t>Surrey Mixed 1</t>
+  </si>
+  <si>
+    <t>Falmer STP Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Queen Mary Mixed 1</t>
+  </si>
+  <si>
+    <t>Chislehurst Sports Ground Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Cambridge Mixed 1</t>
+  </si>
+  <si>
+    <t>Coldhams Common (Abbey Pools), Whitehall Road CB5 8NT Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Anglia Ruskin Mixed 1 (Cambridge)</t>
+  </si>
+  <si>
+    <t>East London Rugby Club Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Chichester Mixed 1</t>
+  </si>
+  <si>
+    <t>Teesside Mixed 1</t>
+  </si>
+  <si>
+    <t>13 - 12</t>
+  </si>
+  <si>
+    <t>Olympia Building Middlesbrough TS1 3BF Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Manchester Met Mixed 1</t>
+  </si>
+  <si>
+    <t>Burnage Rugby Club Varley Park, Battersea Rd, Stockport SK4 3EA Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Burnage Rugby Club Varley Park, Battersea Rd, Stockport SK4 3EA</t>
+  </si>
+  <si>
+    <t>Liverpool John Moores Mixed 1</t>
+  </si>
+  <si>
+    <t>JMO Sports Park Blaguegate Playing Fields Liverpool Road Skelmersdale WN8 8BX Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Bradford Mixed 1</t>
+  </si>
+  <si>
+    <t>University of Bradford Sports Park 3G Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Greenwich Mixed 1</t>
+  </si>
+  <si>
+    <t>Lincoln Mixed 1</t>
+  </si>
+  <si>
+    <t>12 - 47</t>
+  </si>
+  <si>
+    <t>Sheffield Hallam University Sports Park (3G) Provider: BUCS American Football 19-20</t>
+  </si>
+  <si>
+    <t>Edinburgh Napier Mixed 1</t>
   </si>
 </sst>
 </file>
@@ -897,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D36C6C2A-6236-3A41-9DF0-360A3C916FDF}">
-  <dimension ref="A1:A423"/>
+  <dimension ref="A1:A579"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -905,1317 +1202,1317 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>143</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>125</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>122</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>1</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>144</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>1</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>64</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>1</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>1</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>50</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>1</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>1</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>130</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>1</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>145</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>24</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>115</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>1</v>
+        <v>126</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>145</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>26</v>
+        <v>127</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>3</v>
+        <v>128</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>76</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>77</v>
+        <v>129</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>90</v>
+        <v>130</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>140</v>
+        <v>37</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>1</v>
+        <v>132</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>9</v>
+        <v>135</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>90</v>
+        <v>136</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>81</v>
+        <v>137</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>28</v>
+        <v>140</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>90</v>
+        <v>141</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>70</v>
+        <v>114</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>72</v>
+        <v>142</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>73</v>
+        <v>143</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>32</v>
+        <v>144</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>112</v>
+        <v>38</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>56</v>
+        <v>148</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>84</v>
+        <v>149</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>12</v>
+        <v>114</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>14</v>
+        <v>150</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>1</v>
+        <v>95</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>91</v>
+        <v>153</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>42</v>
+        <v>114</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>44</v>
+        <v>154</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>1</v>
+        <v>155</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>122</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>1</v>
+        <v>156</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>1</v>
+        <v>157</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>118</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>66</v>
+        <v>160</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>21</v>
+        <v>161</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>91</v>
+        <v>38</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>95</v>
+        <v>162</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
-        <v>31</v>
+        <v>163</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
-        <v>15</v>
+        <v>165</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
-        <v>91</v>
+        <v>38</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
-        <v>33</v>
+        <v>166</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>118</v>
+        <v>167</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
-        <v>1</v>
+        <v>67</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
-        <v>94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
-        <v>1</v>
+        <v>168</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
-        <v>93</v>
+        <v>169</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
-        <v>122</v>
+        <v>170</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
-        <v>107</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
-        <v>1</v>
+        <v>171</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
-        <v>0</v>
+        <v>114</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
-        <v>108</v>
+        <v>172</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
-        <v>100</v>
+        <v>173</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
-        <v>101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
-        <v>123</v>
+        <v>174</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
-        <v>148</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="s">
-        <v>1</v>
+        <v>175</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
-        <v>55</v>
+        <v>114</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="s">
-        <v>145</v>
+        <v>40</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A206" s="1" t="s">
-        <v>92</v>
+        <v>176</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
-        <v>75</v>
+        <v>177</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="s">
-        <v>40</v>
+        <v>179</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
-        <v>82</v>
+        <v>180</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
-        <v>83</v>
+        <v>181</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
-        <v>123</v>
+        <v>182</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
-        <v>17</v>
+        <v>183</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
-        <v>38</v>
+        <v>185</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
-        <v>19</v>
+        <v>186</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
-        <v>20</v>
+        <v>187</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
-        <v>121</v>
+        <v>0</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
-        <v>22</v>
+        <v>151</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="s">
-        <v>1</v>
+        <v>188</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
-        <v>102</v>
+        <v>0</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
-        <v>1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
-        <v>86</v>
+        <v>189</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="s">
-        <v>151</v>
+        <v>35</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
-        <v>1</v>
+        <v>191</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
-        <v>1</v>
+        <v>85</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="s">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A252" s="1" t="s">
-        <v>131</v>
+        <v>35</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="s">
-        <v>132</v>
+        <v>193</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A254" s="1" t="s">
-        <v>133</v>
+        <v>194</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A257" s="1" t="s">
-        <v>49</v>
+        <v>195</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A258" s="1" t="s">
-        <v>1</v>
+        <v>196</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="s">
-        <v>154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A260" s="1" t="s">
-        <v>1</v>
+        <v>60</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A261" s="1" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A262" s="1" t="s">
-        <v>153</v>
+        <v>197</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A263" s="1" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.2">
@@ -2225,797 +2522,1577 @@
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A265" s="1" t="s">
-        <v>71</v>
+        <v>137</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A266" s="1" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A267" s="1" t="s">
-        <v>1</v>
+        <v>138</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A268" s="1" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A269" s="1" t="s">
-        <v>10</v>
+        <v>195</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A270" s="1" t="s">
-        <v>1</v>
+        <v>198</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="s">
-        <v>137</v>
+        <v>0</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A272" s="1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A273" s="1" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A274" s="1" t="s">
-        <v>153</v>
+        <v>199</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A276" s="1" t="s">
-        <v>119</v>
+        <v>49</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A277" s="1" t="s">
-        <v>120</v>
+        <v>200</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A278" s="1" t="s">
-        <v>78</v>
+        <v>201</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A279" s="1" t="s">
-        <v>1</v>
+        <v>202</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A280" s="1" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A281" s="1" t="s">
-        <v>75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A282" s="1" t="s">
-        <v>1</v>
+        <v>203</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A283" s="1" t="s">
-        <v>155</v>
+        <v>0</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A284" s="1" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A285" s="1" t="s">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A286" s="1" t="s">
-        <v>153</v>
+        <v>204</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="s">
-        <v>117</v>
+        <v>205</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A288" s="1" t="s">
-        <v>82</v>
+        <v>37</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A289" s="1" t="s">
-        <v>83</v>
+        <v>206</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A290" s="1" t="s">
-        <v>1</v>
+        <v>207</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A291" s="1" t="s">
-        <v>121</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A292" s="1" t="s">
-        <v>51</v>
+        <v>195</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A293" s="1" t="s">
-        <v>1</v>
+        <v>208</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A294" s="1" t="s">
-        <v>156</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A295" s="1" t="s">
-        <v>1</v>
+        <v>27</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A296" s="1" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A297" s="1" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A298" s="1" t="s">
-        <v>88</v>
+        <v>205</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A299" s="1" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A300" s="1" t="s">
-        <v>135</v>
+        <v>209</v>
       </c>
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A301" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A302" s="1" t="s">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A303" s="1" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
     </row>
     <row r="304" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A304" s="1" t="s">
-        <v>1</v>
+        <v>210</v>
       </c>
     </row>
     <row r="305" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A305" s="1" t="s">
-        <v>149</v>
+        <v>0</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A306" s="1" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A307" s="1" t="s">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="308" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A308" s="1" t="s">
-        <v>157</v>
+        <v>211</v>
       </c>
     </row>
     <row r="309" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A309" s="1" t="s">
-        <v>91</v>
+        <v>212</v>
       </c>
     </row>
     <row r="310" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A310" s="1" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
     </row>
     <row r="311" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A311" s="1" t="s">
-        <v>68</v>
+        <v>213</v>
       </c>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A312" s="1" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
     </row>
     <row r="313" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A313" s="1" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="314" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A314" s="1" t="s">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A315" s="1" t="s">
-        <v>18</v>
+        <v>151</v>
       </c>
     </row>
     <row r="316" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A316" s="1" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
     </row>
     <row r="317" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A317" s="1" t="s">
-        <v>103</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A318" s="1" t="s">
-        <v>1</v>
+        <v>214</v>
       </c>
     </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A319" s="1" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A320" s="1" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A321" s="1" t="s">
-        <v>91</v>
+        <v>212</v>
       </c>
     </row>
     <row r="322" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A322" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A323" s="1" t="s">
-        <v>27</v>
+        <v>215</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A324" s="1" t="s">
-        <v>1</v>
+        <v>90</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A325" s="1" t="s">
-        <v>118</v>
+        <v>17</v>
       </c>
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A326" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A327" s="1" t="s">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="328" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A328" s="1" t="s">
-        <v>129</v>
+        <v>216</v>
       </c>
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A329" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A330" s="1" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
     </row>
     <row r="331" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A331" s="1" t="s">
-        <v>157</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A332" s="1" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A333" s="1" t="s">
-        <v>119</v>
+        <v>212</v>
       </c>
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A334" s="1" t="s">
-        <v>120</v>
+        <v>37</v>
       </c>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A335" s="1" t="s">
-        <v>78</v>
+        <v>217</v>
       </c>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A336" s="1" t="s">
-        <v>1</v>
+        <v>218</v>
       </c>
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A337" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A338" s="1" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A339" s="1" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="340" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A340" s="1" t="s">
-        <v>47</v>
+        <v>152</v>
       </c>
     </row>
     <row r="341" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A341" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A342" s="1" t="s">
-        <v>8</v>
+        <v>219</v>
       </c>
     </row>
     <row r="343" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A343" s="1" t="s">
-        <v>157</v>
+        <v>0</v>
       </c>
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A344" s="1" t="s">
-        <v>93</v>
+        <v>220</v>
       </c>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A345" s="1" t="s">
-        <v>100</v>
+        <v>212</v>
       </c>
     </row>
     <row r="346" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A346" s="1" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A347" s="1" t="s">
-        <v>1</v>
+        <v>154</v>
       </c>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A348" s="1" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A349" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="350" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A350" s="1" t="s">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="351" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A351" s="1" t="s">
-        <v>127</v>
+        <v>165</v>
       </c>
     </row>
     <row r="352" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A352" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A353" s="1" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
     </row>
     <row r="354" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A354" s="1" t="s">
-        <v>157</v>
+        <v>0</v>
       </c>
     </row>
     <row r="355" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A355" s="1" t="s">
-        <v>92</v>
+        <v>221</v>
       </c>
     </row>
     <row r="356" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A356" s="1" t="s">
-        <v>150</v>
+        <v>212</v>
       </c>
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A357" s="1" t="s">
-        <v>151</v>
+        <v>37</v>
       </c>
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A358" s="1" t="s">
-        <v>152</v>
+        <v>222</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A359" s="1" t="s">
-        <v>1</v>
+        <v>223</v>
       </c>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A360" s="1" t="s">
-        <v>122</v>
+        <v>0</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A361" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A362" s="1" t="s">
-        <v>1</v>
+        <v>175</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A363" s="1" t="s">
-        <v>116</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A364" s="1" t="s">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A365" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="366" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A366" s="1" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
     </row>
     <row r="367" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A367" s="1" t="s">
-        <v>85</v>
+        <v>212</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A368" s="1" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A369" s="1" t="s">
-        <v>63</v>
+        <v>224</v>
       </c>
     </row>
     <row r="370" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A370" s="1" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="371" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A371" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A372" s="1" t="s">
-        <v>118</v>
+        <v>195</v>
       </c>
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A373" s="1" t="s">
-        <v>75</v>
+        <v>199</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A374" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="375" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A375" s="1" t="s">
-        <v>158</v>
+        <v>69</v>
       </c>
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A376" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A377" s="1" t="s">
-        <v>25</v>
+        <v>196</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A378" s="1" t="s">
-        <v>157</v>
+        <v>212</v>
       </c>
     </row>
     <row r="379" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A379" s="1" t="s">
-        <v>117</v>
+        <v>38</v>
       </c>
     </row>
     <row r="380" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A380" s="1" t="s">
-        <v>82</v>
+        <v>225</v>
       </c>
     </row>
     <row r="381" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A381" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A382" s="1" t="s">
-        <v>1</v>
+        <v>226</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A383" s="1" t="s">
-        <v>118</v>
+        <v>0</v>
       </c>
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A384" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A385" s="1" t="s">
-        <v>1</v>
+        <v>227</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A386" s="1" t="s">
-        <v>114</v>
+        <v>0</v>
       </c>
     </row>
     <row r="387" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A387" s="1" t="s">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="388" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A388" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="389" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A389" s="1" t="s">
-        <v>159</v>
+        <v>113</v>
       </c>
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A390" s="1" t="s">
-        <v>86</v>
+        <v>212</v>
       </c>
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A391" s="1" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A392" s="1" t="s">
-        <v>1</v>
+        <v>228</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A393" s="1" t="s">
-        <v>123</v>
+        <v>14</v>
       </c>
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A394" s="1" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A395" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A396" s="1" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
     </row>
     <row r="397" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A397" s="1" t="s">
-        <v>1</v>
+        <v>158</v>
       </c>
     </row>
     <row r="398" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A398" s="1" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="399" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A399" s="1" t="s">
-        <v>159</v>
+        <v>41</v>
       </c>
     </row>
     <row r="400" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A400" s="1" t="s">
-        <v>160</v>
+        <v>0</v>
       </c>
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A401" s="1" t="s">
-        <v>2</v>
+        <v>111</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A402" s="1" t="s">
-        <v>1</v>
+        <v>212</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A403" s="1" t="s">
-        <v>122</v>
+        <v>38</v>
       </c>
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A404" s="1" t="s">
-        <v>36</v>
+        <v>229</v>
       </c>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A405" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A406" s="1" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A407" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A408" s="1" t="s">
-        <v>11</v>
+        <v>118</v>
       </c>
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A409" s="1" t="s">
-        <v>162</v>
+        <v>120</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A410" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A411" s="1" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
     </row>
     <row r="412" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A412" s="1" t="s">
-        <v>121</v>
+        <v>0</v>
       </c>
     </row>
     <row r="413" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A413" s="1" t="s">
-        <v>41</v>
+        <v>230</v>
       </c>
     </row>
     <row r="414" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A414" s="1" t="s">
-        <v>1</v>
+        <v>212</v>
       </c>
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A415" s="1" t="s">
-        <v>104</v>
+        <v>38</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A416" s="1" t="s">
-        <v>1</v>
+        <v>231</v>
       </c>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A417" s="1" t="s">
-        <v>22</v>
+        <v>232</v>
       </c>
     </row>
     <row r="418" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A418" s="1" t="s">
-        <v>162</v>
+        <v>65</v>
       </c>
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A419" s="1" t="s">
-        <v>87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A420" s="1" t="s">
-        <v>52</v>
+        <v>118</v>
       </c>
     </row>
     <row r="421" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A421" s="1" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
     </row>
     <row r="422" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A422" s="1" t="s">
-        <v>54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="423" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A423" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="424" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A424" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A425" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="426" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A426" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="427" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A427" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="428" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A428" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="429" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A429" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="430" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A430" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="431" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A431" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A432" s="1" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="433" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A433" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="434" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A434" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A435" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="436" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A436" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A437" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="438" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A438" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="439" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A439" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="440" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A440" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="441" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A441" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="442" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A442" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A443" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="444" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A444" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="445" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A445" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A446" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="447" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A447" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A448" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="449" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A449" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="450" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A450" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="451" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A451" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A452" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="453" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A453" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A454" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="455" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A455" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="456" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A456" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A457" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="458" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A458" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A459" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="460" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A460" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="461" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A461" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="462" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A462" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="463" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A463" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="464" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A464" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A465" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A466" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A467" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A468" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="469" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A469" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A470" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="471" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A471" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="472" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A472" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="473" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A473" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="474" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A474" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="475" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A475" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="476" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A476" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="477" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A477" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="478" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A478" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A479" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="480" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A480" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A481" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="482" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A482" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="483" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A483" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="484" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A484" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="485" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A485" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="486" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A486" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A487" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="488" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A488" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="489" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A489" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A490" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="491" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A491" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A492" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="493" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A493" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="494" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A494" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="495" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A495" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="496" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A496" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="497" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A497" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="498" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A498" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A499" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="500" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A500" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="501" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A501" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A502" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="503" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A503" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A504" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="505" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A505" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A506" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="507" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A507" s="1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="508" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A508" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="509" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A509" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A510" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="511" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A511" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="512" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A512" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A513" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="514" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A514" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A515" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="516" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A516" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="517" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A517" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A518" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="519" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A519" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="520" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A520" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="521" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A521" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="522" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A522" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A523" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A524" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="525" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A525" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="526" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A526" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="527" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A527" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="528" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A528" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="529" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A529" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="530" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A530" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="531" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A531" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="532" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A532" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A533" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="534" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A534" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="535" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A535" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A536" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="537" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A537" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A538" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="539" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A539" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="540" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A540" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="541" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A541" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="542" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A542" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="543" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A543" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A544" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="545" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A545" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="546" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A546" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A547" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="548" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A548" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A549" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="550" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A550" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="551" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A551" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="552" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A552" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="553" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A553" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="554" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A554" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="555" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A555" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="556" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A556" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="557" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A557" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="558" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A558" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="559" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A559" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="560" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A560" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="561" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A561" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="562" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A562" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="563" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A563" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="564" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A564" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="565" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A565" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="566" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A566" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="567" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A567" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="568" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A568" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="569" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A569" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="570" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A570" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="571" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A571" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="572" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A572" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="573" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A573" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="574" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A574" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="575" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A575" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="576" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A576" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="577" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A577" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="578" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A578" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="579" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A579" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>